<commit_message>
Added Fluffy PET and discrepancy metric between duplicates of each material per CHOL input
</commit_message>
<xml_diff>
--- a/Materials Dataset.xlsx
+++ b/Materials Dataset.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
   <si>
     <t>material</t>
   </si>
@@ -23,36 +23,36 @@
     <t>thickness</t>
   </si>
   <si>
+    <t>surface_productivity_SD</t>
+  </si>
+  <si>
     <t>density</t>
   </si>
   <si>
-    <t>surface_productivity_SD</t>
+    <t>biomass_productivity</t>
   </si>
   <si>
     <t>porosity</t>
   </si>
   <si>
+    <t>biomass_productivity_SD</t>
+  </si>
+  <si>
     <t>moisture_abs</t>
   </si>
   <si>
-    <t>biomass_productivity</t>
-  </si>
-  <si>
     <t>CHOL_input</t>
   </si>
   <si>
-    <t>biomass_productivity_SD</t>
+    <t>product_conc</t>
+  </si>
+  <si>
+    <t>product_conc_SD</t>
   </si>
   <si>
     <t>Poplar</t>
   </si>
   <si>
-    <t>product_conc</t>
-  </si>
-  <si>
-    <t>product_conc_SD</t>
-  </si>
-  <si>
     <t>yield</t>
   </si>
   <si>
@@ -69,12 +69,27 @@
   </si>
   <si>
     <t>Milkweed</t>
+  </si>
+  <si>
+    <t>Viscose</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Porous_PET</t>
+  </si>
+  <si>
+    <t>Fluffy_PET</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <sz val="10.0"/>
@@ -97,12 +112,24 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -111,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -123,6 +150,24 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -353,21 +398,21 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1">
         <v>3.094</v>
@@ -387,7 +432,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>3.094</v>
@@ -407,7 +452,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1">
         <v>3.094</v>
@@ -427,7 +472,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1">
         <v>3.094</v>
@@ -603,6 +648,249 @@
       </c>
       <c r="F13" s="1">
         <v>5.574</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="C14" s="1">
+        <v>60.0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="C15" s="1">
+        <v>60.0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="C16" s="1">
+        <v>60.0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F16" s="4">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="C17" s="1">
+        <v>60.0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F17" s="4">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0.345</v>
+      </c>
+      <c r="C18" s="1">
+        <v>80.0</v>
+      </c>
+      <c r="D18" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F18" s="4">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0.345</v>
+      </c>
+      <c r="C19" s="1">
+        <v>80.0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F19" s="4">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="1">
+        <v>0.345</v>
+      </c>
+      <c r="C20" s="1">
+        <v>80.0</v>
+      </c>
+      <c r="D20" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F20" s="4">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1">
+        <v>0.345</v>
+      </c>
+      <c r="C21" s="1">
+        <v>80.0</v>
+      </c>
+      <c r="D21" s="1">
+        <v>84.0</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F21" s="4">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="C22" s="1">
+        <v>100.0</v>
+      </c>
+      <c r="D22" s="1">
+        <v>87.0</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F22" s="4">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="C23" s="1">
+        <v>100.0</v>
+      </c>
+      <c r="D23" s="1">
+        <v>87.0</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F23" s="4">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="C24" s="1">
+        <v>100.0</v>
+      </c>
+      <c r="D24" s="1">
+        <v>87.0</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F24" s="4">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="C25" s="1">
+        <v>100.0</v>
+      </c>
+      <c r="D25" s="1">
+        <v>87.0</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="F25" s="4">
+        <v>8.0</v>
       </c>
     </row>
   </sheetData>
@@ -626,19 +914,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>13</v>
@@ -1036,6 +1324,382 @@
       <c r="J13" s="3">
         <v>1.761</v>
       </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6">
+        <v>12.8642</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0.6378</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.4608</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0.0371</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0.8135</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0.0513</v>
+      </c>
+      <c r="G14" s="7">
+        <v>81.3507</v>
+      </c>
+      <c r="H14" s="7">
+        <v>5.1345</v>
+      </c>
+      <c r="I14" s="6">
+        <v>24.16696429</v>
+      </c>
+      <c r="J14" s="6">
+        <v>1.602678571</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6">
+        <v>19.6455</v>
+      </c>
+      <c r="B15" s="6">
+        <v>0.9478</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.7055</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0.0821</v>
+      </c>
+      <c r="E15" s="6">
+        <v>1.2337</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0.0649</v>
+      </c>
+      <c r="G15" s="7">
+        <v>61.6863</v>
+      </c>
+      <c r="H15" s="7">
+        <v>3.2452</v>
+      </c>
+      <c r="I15" s="6">
+        <v>24.16696429</v>
+      </c>
+      <c r="J15" s="6">
+        <v>1.602678571</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6">
+        <v>27.9679</v>
+      </c>
+      <c r="B16" s="6">
+        <v>2.4334</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1.0154</v>
+      </c>
+      <c r="D16" s="6">
+        <v>0.1691</v>
+      </c>
+      <c r="E16" s="6">
+        <v>1.8337</v>
+      </c>
+      <c r="F16" s="6">
+        <v>0.1452</v>
+      </c>
+      <c r="G16" s="7">
+        <v>45.8427</v>
+      </c>
+      <c r="H16" s="7">
+        <v>3.63</v>
+      </c>
+      <c r="I16" s="6">
+        <v>24.16696429</v>
+      </c>
+      <c r="J16" s="6">
+        <v>1.602678571</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6">
+        <v>12.4852</v>
+      </c>
+      <c r="B17" s="6">
+        <v>0.8616</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.4459</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.0338</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0.7759</v>
+      </c>
+      <c r="F17" s="6">
+        <v>0.0848</v>
+      </c>
+      <c r="G17" s="7">
+        <v>9.6986</v>
+      </c>
+      <c r="H17" s="7">
+        <v>1.0601</v>
+      </c>
+      <c r="I17" s="6">
+        <v>24.16696429</v>
+      </c>
+      <c r="J17" s="6">
+        <v>1.602678571</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6">
+        <v>14.5768</v>
+      </c>
+      <c r="B18" s="6">
+        <v>0.9013</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.5201</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0.0588</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0.926</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0.0576</v>
+      </c>
+      <c r="G18" s="7">
+        <v>92.5997</v>
+      </c>
+      <c r="H18" s="7">
+        <v>5.7564</v>
+      </c>
+      <c r="I18" s="6">
+        <v>28.57916667</v>
+      </c>
+      <c r="J18" s="6">
+        <v>2.092261905</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6">
+        <v>19.6702</v>
+      </c>
+      <c r="B19" s="6">
+        <v>0.8472</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.6987</v>
+      </c>
+      <c r="D19" s="6">
+        <v>0.069</v>
+      </c>
+      <c r="E19" s="6">
+        <v>1.2282</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0.0655</v>
+      </c>
+      <c r="G19" s="7">
+        <v>61.4121</v>
+      </c>
+      <c r="H19" s="7">
+        <v>3.2765</v>
+      </c>
+      <c r="I19" s="6">
+        <v>28.57916667</v>
+      </c>
+      <c r="J19" s="6">
+        <v>2.092261905</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6">
+        <v>34.3548</v>
+      </c>
+      <c r="B20" s="6">
+        <v>6.9152</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1.2524</v>
+      </c>
+      <c r="D20" s="6">
+        <v>0.3574</v>
+      </c>
+      <c r="E20" s="6">
+        <v>2.2227</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0.4402</v>
+      </c>
+      <c r="G20" s="7">
+        <v>55.5675</v>
+      </c>
+      <c r="H20" s="7">
+        <v>11.0042</v>
+      </c>
+      <c r="I20" s="6">
+        <v>28.57916667</v>
+      </c>
+      <c r="J20" s="6">
+        <v>2.092261905</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6">
+        <v>29.275</v>
+      </c>
+      <c r="B21" s="6">
+        <v>9.2686</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1.0815</v>
+      </c>
+      <c r="D21" s="6">
+        <v>0.4294</v>
+      </c>
+      <c r="E21" s="6">
+        <v>1.9092</v>
+      </c>
+      <c r="F21" s="6">
+        <v>0.6115</v>
+      </c>
+      <c r="G21" s="7">
+        <v>23.865</v>
+      </c>
+      <c r="H21" s="7">
+        <v>7.6442</v>
+      </c>
+      <c r="I21" s="6">
+        <v>28.57916667</v>
+      </c>
+      <c r="J21" s="6">
+        <v>2.092261905</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6">
+        <v>12.0885</v>
+      </c>
+      <c r="B22" s="6">
+        <v>0.8886</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.4244</v>
+      </c>
+      <c r="D22" s="6">
+        <v>0.0312</v>
+      </c>
+      <c r="E22" s="6">
+        <v>0.7462</v>
+      </c>
+      <c r="F22" s="6">
+        <v>0.0549</v>
+      </c>
+      <c r="G22" s="8">
+        <v>74.6202</v>
+      </c>
+      <c r="H22" s="8">
+        <v>5.4853</v>
+      </c>
+      <c r="I22" s="6">
+        <v>28.483125</v>
+      </c>
+      <c r="J22" s="9"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6">
+        <v>23.4839</v>
+      </c>
+      <c r="B23" s="6">
+        <v>0.8578</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.8245</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0.0301</v>
+      </c>
+      <c r="E23" s="6">
+        <v>1.4496</v>
+      </c>
+      <c r="F23" s="6">
+        <v>0.053</v>
+      </c>
+      <c r="G23" s="8">
+        <v>72.4813</v>
+      </c>
+      <c r="H23" s="8">
+        <v>2.6476</v>
+      </c>
+      <c r="I23" s="6">
+        <v>28.483125</v>
+      </c>
+      <c r="J23" s="9"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6">
+        <v>41.8238</v>
+      </c>
+      <c r="B24" s="6">
+        <v>1.8708</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1.4684</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0.0657</v>
+      </c>
+      <c r="E24" s="6">
+        <v>2.5817</v>
+      </c>
+      <c r="F24" s="6">
+        <v>0.1155</v>
+      </c>
+      <c r="G24" s="8">
+        <v>64.5429</v>
+      </c>
+      <c r="H24" s="8">
+        <v>2.887</v>
+      </c>
+      <c r="I24" s="6">
+        <v>28.483125</v>
+      </c>
+      <c r="J24" s="9"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6">
+        <v>37.1211</v>
+      </c>
+      <c r="B25" s="6">
+        <v>6.1203</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1.3033</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0.2149</v>
+      </c>
+      <c r="E25" s="6">
+        <v>2.2914</v>
+      </c>
+      <c r="F25" s="6">
+        <v>0.3778</v>
+      </c>
+      <c r="G25" s="8">
+        <v>28.6429</v>
+      </c>
+      <c r="H25" s="8">
+        <v>4.7224</v>
+      </c>
+      <c r="I25" s="6">
+        <v>28.483125</v>
+      </c>
+      <c r="J25" s="9"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>